<commit_message>
Add edit functionality for words in list and practice mode
</commit_message>
<xml_diff>
--- a/words_list.xlsx
+++ b/words_list.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\todo-app\vocabulary-app\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E9C5BCF9-E6FC-4B11-903F-6ED5E0BF22B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7F6F0CE-DB87-4E9B-8200-3D7B2E6B49B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="23280" windowHeight="14880" xr2:uid="{6C3D62DF-E242-4509-9E86-6FC1D2BFCE95}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="23280" windowHeight="14880" activeTab="1" xr2:uid="{6C3D62DF-E242-4509-9E86-6FC1D2BFCE95}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="152">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="160">
   <si>
     <t>meticulous</t>
   </si>
@@ -495,6 +496,30 @@
   </si>
   <si>
     <t>Words used</t>
+  </si>
+  <si>
+    <t>Github</t>
+  </si>
+  <si>
+    <t>supabase</t>
+  </si>
+  <si>
+    <t>database</t>
+  </si>
+  <si>
+    <t>Render</t>
+  </si>
+  <si>
+    <t>to get domain and run on cloude</t>
+  </si>
+  <si>
+    <t>repository</t>
+  </si>
+  <si>
+    <t>https://console.cloud.google.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Google email sign in </t>
   </si>
 </sst>
 </file>
@@ -1650,4 +1675,49 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{122BCCE3-5263-4B73-8CF3-439FE2AF645F}">
+  <dimension ref="A1:B4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="19.5703125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>155</v>
+      </c>
+      <c r="B1" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>152</v>
+      </c>
+      <c r="B2" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>153</v>
+      </c>
+      <c r="B3" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>159</v>
+      </c>
+      <c r="B4" t="s">
+        <v>158</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>